<commit_message>
Kit v1.1: add register of provisions in motion
One row per status component, with the issuer's source, last resolved,
next check and known pending changes. Example rows re-resolved 2026-10-10.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fd1QFMvYddHhRn3tvR18wb
</commit_message>
<xml_diff>
--- a/kit/citation-provenance-kit.xlsx
+++ b/kit/citation-provenance-kit.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Grades &amp; notation" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Cost calculator" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Example log v1.1" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Register in motion" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -46,13 +47,35 @@
 </comments>
 </file>
 
+<file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="A5" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Grey rows: the domain paper's register, re-resolved on 10 Oct 2026. Overwrite or delete them.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="279">
   <si>
     <t xml:space="preserve">Citation provenance kit — reproduction kit</t>
   </si>
   <si>
-    <t xml:space="preserve">Kit v1.0 · accompanies What Breaks in a Citation, v1.1 (26 July 2026) · CC0 1.0 (no rights reserved)</t>
+    <t xml:space="preserve">Kit v1.1 · accompanies What Breaks in a Citation, v1.1 (26 July 2026) · CC0 1.0 (no rights reserved)</t>
   </si>
   <si>
     <t xml:space="preserve">What this is</t>
@@ -74,7 +97,8 @@
 Components — the ten components and the one sorting question.
 Grades &amp; notation — A–D, the null slot, and the rules for writing them.
 Cost calculator — actions × counts × your own unit times.
-Example log v1.1 — Appendix A of the paper, lightly condensed.</t>
+Example log v1.1 — Appendix A of the paper, lightly condensed.
+Register in motion — status components with an issuer's source and a next-check date (kit v1.1).</t>
   </si>
   <si>
     <t xml:space="preserve">Three rules for the log</t>
@@ -1188,6 +1212,312 @@
   </si>
   <si>
     <t xml:space="preserve">Not in this log: effort (no durations), confirmations (kept elsewhere), and five post-publication defects (the log closed at release).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every status component (commencement, edition, existence, dependency) gets a row, an issuer's source and a next-check date. Record what could move the value, not only the value.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Provision
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">規定</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Component
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">成分</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Value as resolved
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">確認した値</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Grade
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">評価</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Issuer's source (URL)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">発行者の出典</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Last resolved
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">最終確認日</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Next check
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次回確認</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Known pending changes (invalidation events)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">値を動かしうる既知の変化</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Notes
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">備考</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">India — DPDP Rules 2025, Rules 3, 5–16, 22, 23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eighteen months from publication (month: May 2027 — author's arithmetic)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">period: A | still operative: —</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gazette notification G.S.R. 846(E), 13 Nov 2025, Rule 1(4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly; and on any MeitY notification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MeitY sought views (Jan 2026) on cutting 18 months to 12; no amending notification found on 2026-10-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A government explainer (17 Nov 2025) gives the notification date as 14 Nov 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">India — DPDP Rules 2025, Rule 4 (consent managers)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Twelve months from publication (month: November 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G.S.R. 846(E), Rule 1(3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">November 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Japan — Corporate Governance Code (July 2026), English edition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provisional translation available, dated 21 Jul 2026; posting date not shown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exists: A | existed on 24 Jul: —</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.jpx.co.jp/english/equities/listing/cg/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On any change to the page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terms differ from the author's translation: General Principle, Interpretive Guidance, reasonableness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Japan — NTA Q&amp;A on electronic books (books and documents)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">July 2026 edition listed; posting date not shown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exists: A | current on 24 Jul: —</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nta.go.jp/law/joho-zeikaishaku/sonota/jirei/4-3.htm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each June–July</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conflict: a practitioner report (C) says published 10 Jul 2026. Question numbers and pages to be retaken</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Japan — Electronic Books Regulation art. 5(5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Becomes art. 5(4) on 1 Jan 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A (as recorded in the Q&amp;A)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NTA Q&amp;A, definitions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-01</t>
   </si>
 </sst>
 </file>
@@ -1746,7 +2076,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
@@ -6399,4 +6729,881 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I69"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="30"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="I6" s="6"/>
+    </row>
+    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="I9" s="6"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="7"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="7"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="7"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="7"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="7"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="7"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="7"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="7"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="7"/>
+      <c r="B32" s="7"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
+      <c r="G32" s="7"/>
+      <c r="H32" s="7"/>
+      <c r="I32" s="7"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7"/>
+      <c r="B33" s="7"/>
+      <c r="C33" s="7"/>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="7"/>
+      <c r="H33" s="7"/>
+      <c r="I33" s="7"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="7"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="7"/>
+      <c r="B36" s="7"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="7"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="7"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7"/>
+      <c r="B38" s="7"/>
+      <c r="C38" s="7"/>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="7"/>
+      <c r="H38" s="7"/>
+      <c r="I38" s="7"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7"/>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
+      <c r="H39" s="7"/>
+      <c r="I39" s="7"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7"/>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="7"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7"/>
+      <c r="B41" s="7"/>
+      <c r="C41" s="7"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="7"/>
+      <c r="H41" s="7"/>
+      <c r="I41" s="7"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7"/>
+      <c r="B42" s="7"/>
+      <c r="C42" s="7"/>
+      <c r="D42" s="7"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="7"/>
+      <c r="G42" s="7"/>
+      <c r="H42" s="7"/>
+      <c r="I42" s="7"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="7"/>
+      <c r="B43" s="7"/>
+      <c r="C43" s="7"/>
+      <c r="D43" s="7"/>
+      <c r="E43" s="7"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="7"/>
+      <c r="H43" s="7"/>
+      <c r="I43" s="7"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="7"/>
+      <c r="B44" s="7"/>
+      <c r="C44" s="7"/>
+      <c r="D44" s="7"/>
+      <c r="E44" s="7"/>
+      <c r="F44" s="7"/>
+      <c r="G44" s="7"/>
+      <c r="H44" s="7"/>
+      <c r="I44" s="7"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="7"/>
+      <c r="B45" s="7"/>
+      <c r="C45" s="7"/>
+      <c r="D45" s="7"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="7"/>
+      <c r="I45" s="7"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="7"/>
+      <c r="B46" s="7"/>
+      <c r="C46" s="7"/>
+      <c r="D46" s="7"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="7"/>
+      <c r="G46" s="7"/>
+      <c r="H46" s="7"/>
+      <c r="I46" s="7"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="7"/>
+      <c r="B47" s="7"/>
+      <c r="C47" s="7"/>
+      <c r="D47" s="7"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="7"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="7"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="7"/>
+      <c r="B48" s="7"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="7"/>
+      <c r="I48" s="7"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="7"/>
+      <c r="B49" s="7"/>
+      <c r="C49" s="7"/>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="7"/>
+      <c r="I49" s="7"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="7"/>
+      <c r="B50" s="7"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
+      <c r="H50" s="7"/>
+      <c r="I50" s="7"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="7"/>
+      <c r="B51" s="7"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="7"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="7"/>
+      <c r="B52" s="7"/>
+      <c r="C52" s="7"/>
+      <c r="D52" s="7"/>
+      <c r="E52" s="7"/>
+      <c r="F52" s="7"/>
+      <c r="G52" s="7"/>
+      <c r="H52" s="7"/>
+      <c r="I52" s="7"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="7"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7"/>
+      <c r="G53" s="7"/>
+      <c r="H53" s="7"/>
+      <c r="I53" s="7"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7"/>
+      <c r="B54" s="7"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="7"/>
+      <c r="G54" s="7"/>
+      <c r="H54" s="7"/>
+      <c r="I54" s="7"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="7"/>
+      <c r="B55" s="7"/>
+      <c r="C55" s="7"/>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="7"/>
+      <c r="G55" s="7"/>
+      <c r="H55" s="7"/>
+      <c r="I55" s="7"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="7"/>
+      <c r="B56" s="7"/>
+      <c r="C56" s="7"/>
+      <c r="D56" s="7"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="7"/>
+      <c r="G56" s="7"/>
+      <c r="H56" s="7"/>
+      <c r="I56" s="7"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="7"/>
+      <c r="B57" s="7"/>
+      <c r="C57" s="7"/>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="7"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="7"/>
+      <c r="I57" s="7"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="7"/>
+      <c r="B58" s="7"/>
+      <c r="C58" s="7"/>
+      <c r="D58" s="7"/>
+      <c r="E58" s="7"/>
+      <c r="F58" s="7"/>
+      <c r="G58" s="7"/>
+      <c r="H58" s="7"/>
+      <c r="I58" s="7"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="7"/>
+      <c r="B59" s="7"/>
+      <c r="C59" s="7"/>
+      <c r="D59" s="7"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="7"/>
+      <c r="G59" s="7"/>
+      <c r="H59" s="7"/>
+      <c r="I59" s="7"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="7"/>
+      <c r="B60" s="7"/>
+      <c r="C60" s="7"/>
+      <c r="D60" s="7"/>
+      <c r="E60" s="7"/>
+      <c r="F60" s="7"/>
+      <c r="G60" s="7"/>
+      <c r="H60" s="7"/>
+      <c r="I60" s="7"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="7"/>
+      <c r="B61" s="7"/>
+      <c r="C61" s="7"/>
+      <c r="D61" s="7"/>
+      <c r="E61" s="7"/>
+      <c r="F61" s="7"/>
+      <c r="G61" s="7"/>
+      <c r="H61" s="7"/>
+      <c r="I61" s="7"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="7"/>
+      <c r="B62" s="7"/>
+      <c r="C62" s="7"/>
+      <c r="D62" s="7"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="7"/>
+      <c r="G62" s="7"/>
+      <c r="H62" s="7"/>
+      <c r="I62" s="7"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="7"/>
+      <c r="B63" s="7"/>
+      <c r="C63" s="7"/>
+      <c r="D63" s="7"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="7"/>
+      <c r="G63" s="7"/>
+      <c r="H63" s="7"/>
+      <c r="I63" s="7"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="7"/>
+      <c r="B64" s="7"/>
+      <c r="C64" s="7"/>
+      <c r="D64" s="7"/>
+      <c r="E64" s="7"/>
+      <c r="F64" s="7"/>
+      <c r="G64" s="7"/>
+      <c r="H64" s="7"/>
+      <c r="I64" s="7"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="7"/>
+      <c r="B65" s="7"/>
+      <c r="C65" s="7"/>
+      <c r="D65" s="7"/>
+      <c r="E65" s="7"/>
+      <c r="F65" s="7"/>
+      <c r="G65" s="7"/>
+      <c r="H65" s="7"/>
+      <c r="I65" s="7"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="7"/>
+      <c r="B66" s="7"/>
+      <c r="C66" s="7"/>
+      <c r="D66" s="7"/>
+      <c r="E66" s="7"/>
+      <c r="F66" s="7"/>
+      <c r="G66" s="7"/>
+      <c r="H66" s="7"/>
+      <c r="I66" s="7"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="7"/>
+      <c r="B67" s="7"/>
+      <c r="C67" s="7"/>
+      <c r="D67" s="7"/>
+      <c r="E67" s="7"/>
+      <c r="F67" s="7"/>
+      <c r="G67" s="7"/>
+      <c r="H67" s="7"/>
+      <c r="I67" s="7"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="7"/>
+      <c r="B68" s="7"/>
+      <c r="C68" s="7"/>
+      <c r="D68" s="7"/>
+      <c r="E68" s="7"/>
+      <c r="F68" s="7"/>
+      <c r="G68" s="7"/>
+      <c r="H68" s="7"/>
+      <c r="I68" s="7"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="7"/>
+      <c r="B69" s="7"/>
+      <c r="C69" s="7"/>
+      <c r="D69" s="7"/>
+      <c r="E69" s="7"/>
+      <c r="F69" s="7"/>
+      <c r="G69" s="7"/>
+      <c r="H69" s="7"/>
+      <c r="I69" s="7"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B200" type="list">
+      <formula1>Components!$A$5:$A$20</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Kit v1.8 (unreleased): catchlog --fields, who-wrote column, workbook text fixes, series log example
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C2RNJLwLc4CBTFwfe5m9zY
</commit_message>
<xml_diff>
--- a/kit/citation-provenance-kit.xlsx
+++ b/kit/citation-provenance-kit.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
@@ -42,13 +42,34 @@
           <t xml:space="preserve">Example row drawn from entry #8 of the paper's log. Overwrite or delete it.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>35</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>90</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>21</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
@@ -64,18 +85,39 @@
           <t xml:space="preserve">Grey rows: the domain paper's register, re-resolved on 10 Oct 2026. Overwrite or delete them.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>1</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>24</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="281">
   <si>
     <t xml:space="preserve">Citation provenance kit — reproduction kit</t>
   </si>
   <si>
-    <t xml:space="preserve">Kit v1.1 · accompanies What Breaks in a Citation, v1.1 (26 July 2026) · CC0 1.0 (no rights reserved)</t>
+    <t xml:space="preserve">Kit v1.8 · accompanies What Breaks in a Citation, v1.1 (26 July 2026) · CC0 1.0 (no rights reserved)</t>
   </si>
   <si>
     <t xml:space="preserve">What this is</t>
@@ -105,17 +147,19 @@
   </si>
   <si>
     <t xml:space="preserve">1. Record confirmations and abstentions, not only corrections. Without them there is no denominator.
-2. Fill the 'what would have happened' column yourself. It is the one field nobody else can fill.
+2. Fill the 'what would have happened' column yourself. It is the one field nobody else can fill. If an assistant drafted it, or you chose from its options, say so in the 'Who wrote' column (kit v1.8).
 3. Keep the log open after release. Publication is a marker in the log, not its end.</t>
   </si>
   <si>
     <t xml:space="preserve">Columns the original log lacked</t>
   </si>
   <si>
-    <t xml:space="preserve">'Did an existing rule fire?': two rules failed to prevent their own failure from recurring, and the log could not show it (Appendix B, §9-1).
+    <t xml:space="preserve">The original log kept three things for each entry: what was wrong, what was right, and how it came to notice (Appendix A-0). Every other column here was added afterwards. The paper says the six fields of §7-1 were recorded for each correction (§7-1, §8-1); the published log (Appendix A-2, A-6) shows no 'what would have happened' column.
+'Did an existing rule fire?': two rules failed to prevent their own failure from recurring, and the log could not show it (Appendix B, §9-1).
 'Duration': no effort was recorded and it cannot be reconstructed (§8-1).
 'Stakes': the distinction between a step of the argument collapsing and one footnote dying (§7-1), as a filterable field.
-'Phase': the log closed at release, so post-publication defects went unnumbered (§9-7).</t>
+'Phase': the log closed at release, so post-publication defects went unnumbered (§9-7).
+'Who wrote what would have happened?': the field cannot be delegated (§9-5), so record when it was drafted by an assistant or chosen from an assistant's options (kit v1.8).</t>
   </si>
   <si>
     <t xml:space="preserve">What this kit does not do</t>
@@ -140,7 +184,7 @@
     <t xml:space="preserve">Catch log</t>
   </si>
   <si>
-    <t xml:space="preserve">One row per correction, confirmation or abstention. The seven fields of §10-4, plus four the original log lacked: date found, whether an existing rule fired, stakes (§7-1) and phase (§9-7).</t>
+    <t xml:space="preserve">One row per correction, confirmation or abstention. The seven fields of §10-4, and five more: date found, whether an existing rule fired, stakes (the distinction of §7-1), who wrote the 'what would have happened' field (§9-5), and phase (§9-7).</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -371,6 +415,30 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">Who wrote 'what would have happened'?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">「見逃していたら」を誰が書いたか</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">Duration (minutes)
 </t>
     </r>
@@ -438,6 +506,9 @@
   </si>
   <si>
     <t xml:space="preserve">A step of the argument collapses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">author</t>
   </si>
   <si>
     <t xml:space="preserve">Pre-release</t>
@@ -2084,7 +2155,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
@@ -2092,7 +2163,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="225" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
@@ -2140,7 +2211,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L205"/>
+  <dimension ref="A1:M205"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -2152,8 +2223,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2203,41 +2275,47 @@
       <c r="L4" s="5" t="s">
         <v>31</v>
       </c>
+      <c r="M4" s="5" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6" t="s">
         <v>42</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2255,6 +2333,7 @@
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>
       <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
@@ -2271,6 +2350,7 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
@@ -2287,6 +2367,7 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
@@ -2303,6 +2384,7 @@
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
       <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
@@ -2319,6 +2401,7 @@
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="n">
@@ -2335,6 +2418,7 @@
       <c r="J11" s="7"/>
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
@@ -2351,6 +2435,7 @@
       <c r="J12" s="7"/>
       <c r="K12" s="7"/>
       <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="n">
@@ -2367,6 +2452,7 @@
       <c r="J13" s="7"/>
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="n">
@@ -2383,6 +2469,7 @@
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
       <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="n">
@@ -2399,6 +2486,7 @@
       <c r="J15" s="7"/>
       <c r="K15" s="7"/>
       <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="n">
@@ -2415,6 +2503,7 @@
       <c r="J16" s="7"/>
       <c r="K16" s="7"/>
       <c r="L16" s="7"/>
+      <c r="M16" s="7"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="n">
@@ -2431,6 +2520,7 @@
       <c r="J17" s="7"/>
       <c r="K17" s="7"/>
       <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="n">
@@ -2447,6 +2537,7 @@
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
       <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="n">
@@ -2463,6 +2554,7 @@
       <c r="J19" s="7"/>
       <c r="K19" s="7"/>
       <c r="L19" s="7"/>
+      <c r="M19" s="7"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="n">
@@ -2479,6 +2571,7 @@
       <c r="J20" s="7"/>
       <c r="K20" s="7"/>
       <c r="L20" s="7"/>
+      <c r="M20" s="7"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="n">
@@ -2495,6 +2588,7 @@
       <c r="J21" s="7"/>
       <c r="K21" s="7"/>
       <c r="L21" s="7"/>
+      <c r="M21" s="7"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="n">
@@ -2511,6 +2605,7 @@
       <c r="J22" s="7"/>
       <c r="K22" s="7"/>
       <c r="L22" s="7"/>
+      <c r="M22" s="7"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="n">
@@ -2527,6 +2622,7 @@
       <c r="J23" s="7"/>
       <c r="K23" s="7"/>
       <c r="L23" s="7"/>
+      <c r="M23" s="7"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="n">
@@ -2543,6 +2639,7 @@
       <c r="J24" s="7"/>
       <c r="K24" s="7"/>
       <c r="L24" s="7"/>
+      <c r="M24" s="7"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="n">
@@ -2559,6 +2656,7 @@
       <c r="J25" s="7"/>
       <c r="K25" s="7"/>
       <c r="L25" s="7"/>
+      <c r="M25" s="7"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="n">
@@ -2575,6 +2673,7 @@
       <c r="J26" s="7"/>
       <c r="K26" s="7"/>
       <c r="L26" s="7"/>
+      <c r="M26" s="7"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="n">
@@ -2591,6 +2690,7 @@
       <c r="J27" s="7"/>
       <c r="K27" s="7"/>
       <c r="L27" s="7"/>
+      <c r="M27" s="7"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="n">
@@ -2607,6 +2707,7 @@
       <c r="J28" s="7"/>
       <c r="K28" s="7"/>
       <c r="L28" s="7"/>
+      <c r="M28" s="7"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="n">
@@ -2623,6 +2724,7 @@
       <c r="J29" s="7"/>
       <c r="K29" s="7"/>
       <c r="L29" s="7"/>
+      <c r="M29" s="7"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="n">
@@ -2639,6 +2741,7 @@
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
       <c r="L30" s="7"/>
+      <c r="M30" s="7"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="n">
@@ -2655,6 +2758,7 @@
       <c r="J31" s="7"/>
       <c r="K31" s="7"/>
       <c r="L31" s="7"/>
+      <c r="M31" s="7"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="n">
@@ -2671,6 +2775,7 @@
       <c r="J32" s="7"/>
       <c r="K32" s="7"/>
       <c r="L32" s="7"/>
+      <c r="M32" s="7"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="n">
@@ -2687,6 +2792,7 @@
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
       <c r="L33" s="7"/>
+      <c r="M33" s="7"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="n">
@@ -2703,6 +2809,7 @@
       <c r="J34" s="7"/>
       <c r="K34" s="7"/>
       <c r="L34" s="7"/>
+      <c r="M34" s="7"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="n">
@@ -2719,6 +2826,7 @@
       <c r="J35" s="7"/>
       <c r="K35" s="7"/>
       <c r="L35" s="7"/>
+      <c r="M35" s="7"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="n">
@@ -2735,6 +2843,7 @@
       <c r="J36" s="7"/>
       <c r="K36" s="7"/>
       <c r="L36" s="7"/>
+      <c r="M36" s="7"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="n">
@@ -2751,6 +2860,7 @@
       <c r="J37" s="7"/>
       <c r="K37" s="7"/>
       <c r="L37" s="7"/>
+      <c r="M37" s="7"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="n">
@@ -2767,6 +2877,7 @@
       <c r="J38" s="7"/>
       <c r="K38" s="7"/>
       <c r="L38" s="7"/>
+      <c r="M38" s="7"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="n">
@@ -2783,6 +2894,7 @@
       <c r="J39" s="7"/>
       <c r="K39" s="7"/>
       <c r="L39" s="7"/>
+      <c r="M39" s="7"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="n">
@@ -2799,6 +2911,7 @@
       <c r="J40" s="7"/>
       <c r="K40" s="7"/>
       <c r="L40" s="7"/>
+      <c r="M40" s="7"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="n">
@@ -2815,6 +2928,7 @@
       <c r="J41" s="7"/>
       <c r="K41" s="7"/>
       <c r="L41" s="7"/>
+      <c r="M41" s="7"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="n">
@@ -2831,6 +2945,7 @@
       <c r="J42" s="7"/>
       <c r="K42" s="7"/>
       <c r="L42" s="7"/>
+      <c r="M42" s="7"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="n">
@@ -2847,6 +2962,7 @@
       <c r="J43" s="7"/>
       <c r="K43" s="7"/>
       <c r="L43" s="7"/>
+      <c r="M43" s="7"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="n">
@@ -2863,6 +2979,7 @@
       <c r="J44" s="7"/>
       <c r="K44" s="7"/>
       <c r="L44" s="7"/>
+      <c r="M44" s="7"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="n">
@@ -2879,6 +2996,7 @@
       <c r="J45" s="7"/>
       <c r="K45" s="7"/>
       <c r="L45" s="7"/>
+      <c r="M45" s="7"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="n">
@@ -2895,6 +3013,7 @@
       <c r="J46" s="7"/>
       <c r="K46" s="7"/>
       <c r="L46" s="7"/>
+      <c r="M46" s="7"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="n">
@@ -2911,6 +3030,7 @@
       <c r="J47" s="7"/>
       <c r="K47" s="7"/>
       <c r="L47" s="7"/>
+      <c r="M47" s="7"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="n">
@@ -2927,6 +3047,7 @@
       <c r="J48" s="7"/>
       <c r="K48" s="7"/>
       <c r="L48" s="7"/>
+      <c r="M48" s="7"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="n">
@@ -2943,6 +3064,7 @@
       <c r="J49" s="7"/>
       <c r="K49" s="7"/>
       <c r="L49" s="7"/>
+      <c r="M49" s="7"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="n">
@@ -2959,6 +3081,7 @@
       <c r="J50" s="7"/>
       <c r="K50" s="7"/>
       <c r="L50" s="7"/>
+      <c r="M50" s="7"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="n">
@@ -2975,6 +3098,7 @@
       <c r="J51" s="7"/>
       <c r="K51" s="7"/>
       <c r="L51" s="7"/>
+      <c r="M51" s="7"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="n">
@@ -2991,6 +3115,7 @@
       <c r="J52" s="7"/>
       <c r="K52" s="7"/>
       <c r="L52" s="7"/>
+      <c r="M52" s="7"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="n">
@@ -3007,6 +3132,7 @@
       <c r="J53" s="7"/>
       <c r="K53" s="7"/>
       <c r="L53" s="7"/>
+      <c r="M53" s="7"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="n">
@@ -3023,6 +3149,7 @@
       <c r="J54" s="7"/>
       <c r="K54" s="7"/>
       <c r="L54" s="7"/>
+      <c r="M54" s="7"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="n">
@@ -3039,6 +3166,7 @@
       <c r="J55" s="7"/>
       <c r="K55" s="7"/>
       <c r="L55" s="7"/>
+      <c r="M55" s="7"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="n">
@@ -3055,6 +3183,7 @@
       <c r="J56" s="7"/>
       <c r="K56" s="7"/>
       <c r="L56" s="7"/>
+      <c r="M56" s="7"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="n">
@@ -3071,6 +3200,7 @@
       <c r="J57" s="7"/>
       <c r="K57" s="7"/>
       <c r="L57" s="7"/>
+      <c r="M57" s="7"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="n">
@@ -3087,6 +3217,7 @@
       <c r="J58" s="7"/>
       <c r="K58" s="7"/>
       <c r="L58" s="7"/>
+      <c r="M58" s="7"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="n">
@@ -3103,6 +3234,7 @@
       <c r="J59" s="7"/>
       <c r="K59" s="7"/>
       <c r="L59" s="7"/>
+      <c r="M59" s="7"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="n">
@@ -3119,6 +3251,7 @@
       <c r="J60" s="7"/>
       <c r="K60" s="7"/>
       <c r="L60" s="7"/>
+      <c r="M60" s="7"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="n">
@@ -3135,6 +3268,7 @@
       <c r="J61" s="7"/>
       <c r="K61" s="7"/>
       <c r="L61" s="7"/>
+      <c r="M61" s="7"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="n">
@@ -3151,6 +3285,7 @@
       <c r="J62" s="7"/>
       <c r="K62" s="7"/>
       <c r="L62" s="7"/>
+      <c r="M62" s="7"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="n">
@@ -3167,6 +3302,7 @@
       <c r="J63" s="7"/>
       <c r="K63" s="7"/>
       <c r="L63" s="7"/>
+      <c r="M63" s="7"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="n">
@@ -3183,6 +3319,7 @@
       <c r="J64" s="7"/>
       <c r="K64" s="7"/>
       <c r="L64" s="7"/>
+      <c r="M64" s="7"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="n">
@@ -3199,6 +3336,7 @@
       <c r="J65" s="7"/>
       <c r="K65" s="7"/>
       <c r="L65" s="7"/>
+      <c r="M65" s="7"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="n">
@@ -3215,6 +3353,7 @@
       <c r="J66" s="7"/>
       <c r="K66" s="7"/>
       <c r="L66" s="7"/>
+      <c r="M66" s="7"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="n">
@@ -3231,6 +3370,7 @@
       <c r="J67" s="7"/>
       <c r="K67" s="7"/>
       <c r="L67" s="7"/>
+      <c r="M67" s="7"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="4" t="n">
@@ -3247,6 +3387,7 @@
       <c r="J68" s="7"/>
       <c r="K68" s="7"/>
       <c r="L68" s="7"/>
+      <c r="M68" s="7"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="4" t="n">
@@ -3263,6 +3404,7 @@
       <c r="J69" s="7"/>
       <c r="K69" s="7"/>
       <c r="L69" s="7"/>
+      <c r="M69" s="7"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="4" t="n">
@@ -3279,6 +3421,7 @@
       <c r="J70" s="7"/>
       <c r="K70" s="7"/>
       <c r="L70" s="7"/>
+      <c r="M70" s="7"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="n">
@@ -3295,6 +3438,7 @@
       <c r="J71" s="7"/>
       <c r="K71" s="7"/>
       <c r="L71" s="7"/>
+      <c r="M71" s="7"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="4" t="n">
@@ -3311,6 +3455,7 @@
       <c r="J72" s="7"/>
       <c r="K72" s="7"/>
       <c r="L72" s="7"/>
+      <c r="M72" s="7"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="4" t="n">
@@ -3327,6 +3472,7 @@
       <c r="J73" s="7"/>
       <c r="K73" s="7"/>
       <c r="L73" s="7"/>
+      <c r="M73" s="7"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="4" t="n">
@@ -3343,6 +3489,7 @@
       <c r="J74" s="7"/>
       <c r="K74" s="7"/>
       <c r="L74" s="7"/>
+      <c r="M74" s="7"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="4" t="n">
@@ -3359,6 +3506,7 @@
       <c r="J75" s="7"/>
       <c r="K75" s="7"/>
       <c r="L75" s="7"/>
+      <c r="M75" s="7"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="4" t="n">
@@ -3375,6 +3523,7 @@
       <c r="J76" s="7"/>
       <c r="K76" s="7"/>
       <c r="L76" s="7"/>
+      <c r="M76" s="7"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="n">
@@ -3391,6 +3540,7 @@
       <c r="J77" s="7"/>
       <c r="K77" s="7"/>
       <c r="L77" s="7"/>
+      <c r="M77" s="7"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="4" t="n">
@@ -3407,6 +3557,7 @@
       <c r="J78" s="7"/>
       <c r="K78" s="7"/>
       <c r="L78" s="7"/>
+      <c r="M78" s="7"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="4" t="n">
@@ -3423,6 +3574,7 @@
       <c r="J79" s="7"/>
       <c r="K79" s="7"/>
       <c r="L79" s="7"/>
+      <c r="M79" s="7"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="4" t="n">
@@ -3439,6 +3591,7 @@
       <c r="J80" s="7"/>
       <c r="K80" s="7"/>
       <c r="L80" s="7"/>
+      <c r="M80" s="7"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="4" t="n">
@@ -3455,6 +3608,7 @@
       <c r="J81" s="7"/>
       <c r="K81" s="7"/>
       <c r="L81" s="7"/>
+      <c r="M81" s="7"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="4" t="n">
@@ -3471,6 +3625,7 @@
       <c r="J82" s="7"/>
       <c r="K82" s="7"/>
       <c r="L82" s="7"/>
+      <c r="M82" s="7"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="4" t="n">
@@ -3487,6 +3642,7 @@
       <c r="J83" s="7"/>
       <c r="K83" s="7"/>
       <c r="L83" s="7"/>
+      <c r="M83" s="7"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="4" t="n">
@@ -3503,6 +3659,7 @@
       <c r="J84" s="7"/>
       <c r="K84" s="7"/>
       <c r="L84" s="7"/>
+      <c r="M84" s="7"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="4" t="n">
@@ -3519,6 +3676,7 @@
       <c r="J85" s="7"/>
       <c r="K85" s="7"/>
       <c r="L85" s="7"/>
+      <c r="M85" s="7"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="4" t="n">
@@ -3535,6 +3693,7 @@
       <c r="J86" s="7"/>
       <c r="K86" s="7"/>
       <c r="L86" s="7"/>
+      <c r="M86" s="7"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="4" t="n">
@@ -3551,6 +3710,7 @@
       <c r="J87" s="7"/>
       <c r="K87" s="7"/>
       <c r="L87" s="7"/>
+      <c r="M87" s="7"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="4" t="n">
@@ -3567,6 +3727,7 @@
       <c r="J88" s="7"/>
       <c r="K88" s="7"/>
       <c r="L88" s="7"/>
+      <c r="M88" s="7"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="4" t="n">
@@ -3583,6 +3744,7 @@
       <c r="J89" s="7"/>
       <c r="K89" s="7"/>
       <c r="L89" s="7"/>
+      <c r="M89" s="7"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="4" t="n">
@@ -3599,6 +3761,7 @@
       <c r="J90" s="7"/>
       <c r="K90" s="7"/>
       <c r="L90" s="7"/>
+      <c r="M90" s="7"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="4" t="n">
@@ -3615,6 +3778,7 @@
       <c r="J91" s="7"/>
       <c r="K91" s="7"/>
       <c r="L91" s="7"/>
+      <c r="M91" s="7"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="4" t="n">
@@ -3631,6 +3795,7 @@
       <c r="J92" s="7"/>
       <c r="K92" s="7"/>
       <c r="L92" s="7"/>
+      <c r="M92" s="7"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="4" t="n">
@@ -3647,6 +3812,7 @@
       <c r="J93" s="7"/>
       <c r="K93" s="7"/>
       <c r="L93" s="7"/>
+      <c r="M93" s="7"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="4" t="n">
@@ -3663,6 +3829,7 @@
       <c r="J94" s="7"/>
       <c r="K94" s="7"/>
       <c r="L94" s="7"/>
+      <c r="M94" s="7"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="4" t="n">
@@ -3679,6 +3846,7 @@
       <c r="J95" s="7"/>
       <c r="K95" s="7"/>
       <c r="L95" s="7"/>
+      <c r="M95" s="7"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="4" t="n">
@@ -3695,6 +3863,7 @@
       <c r="J96" s="7"/>
       <c r="K96" s="7"/>
       <c r="L96" s="7"/>
+      <c r="M96" s="7"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="4" t="n">
@@ -3711,6 +3880,7 @@
       <c r="J97" s="7"/>
       <c r="K97" s="7"/>
       <c r="L97" s="7"/>
+      <c r="M97" s="7"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="4" t="n">
@@ -3727,6 +3897,7 @@
       <c r="J98" s="7"/>
       <c r="K98" s="7"/>
       <c r="L98" s="7"/>
+      <c r="M98" s="7"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="4" t="n">
@@ -3743,6 +3914,7 @@
       <c r="J99" s="7"/>
       <c r="K99" s="7"/>
       <c r="L99" s="7"/>
+      <c r="M99" s="7"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="4" t="n">
@@ -3759,6 +3931,7 @@
       <c r="J100" s="7"/>
       <c r="K100" s="7"/>
       <c r="L100" s="7"/>
+      <c r="M100" s="7"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="4" t="n">
@@ -3775,6 +3948,7 @@
       <c r="J101" s="7"/>
       <c r="K101" s="7"/>
       <c r="L101" s="7"/>
+      <c r="M101" s="7"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="4" t="n">
@@ -3791,6 +3965,7 @@
       <c r="J102" s="7"/>
       <c r="K102" s="7"/>
       <c r="L102" s="7"/>
+      <c r="M102" s="7"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="4" t="n">
@@ -3807,6 +3982,7 @@
       <c r="J103" s="7"/>
       <c r="K103" s="7"/>
       <c r="L103" s="7"/>
+      <c r="M103" s="7"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="4" t="n">
@@ -3823,6 +3999,7 @@
       <c r="J104" s="7"/>
       <c r="K104" s="7"/>
       <c r="L104" s="7"/>
+      <c r="M104" s="7"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="4" t="n">
@@ -3839,6 +4016,7 @@
       <c r="J105" s="7"/>
       <c r="K105" s="7"/>
       <c r="L105" s="7"/>
+      <c r="M105" s="7"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="4" t="n">
@@ -3855,6 +4033,7 @@
       <c r="J106" s="7"/>
       <c r="K106" s="7"/>
       <c r="L106" s="7"/>
+      <c r="M106" s="7"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="4" t="n">
@@ -3871,6 +4050,7 @@
       <c r="J107" s="7"/>
       <c r="K107" s="7"/>
       <c r="L107" s="7"/>
+      <c r="M107" s="7"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="4" t="n">
@@ -3887,6 +4067,7 @@
       <c r="J108" s="7"/>
       <c r="K108" s="7"/>
       <c r="L108" s="7"/>
+      <c r="M108" s="7"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="4" t="n">
@@ -3903,6 +4084,7 @@
       <c r="J109" s="7"/>
       <c r="K109" s="7"/>
       <c r="L109" s="7"/>
+      <c r="M109" s="7"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="4" t="n">
@@ -3919,6 +4101,7 @@
       <c r="J110" s="7"/>
       <c r="K110" s="7"/>
       <c r="L110" s="7"/>
+      <c r="M110" s="7"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="4" t="n">
@@ -3935,6 +4118,7 @@
       <c r="J111" s="7"/>
       <c r="K111" s="7"/>
       <c r="L111" s="7"/>
+      <c r="M111" s="7"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="4" t="n">
@@ -3951,6 +4135,7 @@
       <c r="J112" s="7"/>
       <c r="K112" s="7"/>
       <c r="L112" s="7"/>
+      <c r="M112" s="7"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="4" t="n">
@@ -3967,6 +4152,7 @@
       <c r="J113" s="7"/>
       <c r="K113" s="7"/>
       <c r="L113" s="7"/>
+      <c r="M113" s="7"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="4" t="n">
@@ -3983,6 +4169,7 @@
       <c r="J114" s="7"/>
       <c r="K114" s="7"/>
       <c r="L114" s="7"/>
+      <c r="M114" s="7"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="4" t="n">
@@ -3999,6 +4186,7 @@
       <c r="J115" s="7"/>
       <c r="K115" s="7"/>
       <c r="L115" s="7"/>
+      <c r="M115" s="7"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="4" t="n">
@@ -4015,6 +4203,7 @@
       <c r="J116" s="7"/>
       <c r="K116" s="7"/>
       <c r="L116" s="7"/>
+      <c r="M116" s="7"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="4" t="n">
@@ -4031,6 +4220,7 @@
       <c r="J117" s="7"/>
       <c r="K117" s="7"/>
       <c r="L117" s="7"/>
+      <c r="M117" s="7"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="4" t="n">
@@ -4047,6 +4237,7 @@
       <c r="J118" s="7"/>
       <c r="K118" s="7"/>
       <c r="L118" s="7"/>
+      <c r="M118" s="7"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="4" t="n">
@@ -4063,6 +4254,7 @@
       <c r="J119" s="7"/>
       <c r="K119" s="7"/>
       <c r="L119" s="7"/>
+      <c r="M119" s="7"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="4" t="n">
@@ -4079,6 +4271,7 @@
       <c r="J120" s="7"/>
       <c r="K120" s="7"/>
       <c r="L120" s="7"/>
+      <c r="M120" s="7"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="4" t="n">
@@ -4095,6 +4288,7 @@
       <c r="J121" s="7"/>
       <c r="K121" s="7"/>
       <c r="L121" s="7"/>
+      <c r="M121" s="7"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="4" t="n">
@@ -4111,6 +4305,7 @@
       <c r="J122" s="7"/>
       <c r="K122" s="7"/>
       <c r="L122" s="7"/>
+      <c r="M122" s="7"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="4" t="n">
@@ -4127,6 +4322,7 @@
       <c r="J123" s="7"/>
       <c r="K123" s="7"/>
       <c r="L123" s="7"/>
+      <c r="M123" s="7"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="4" t="n">
@@ -4143,6 +4339,7 @@
       <c r="J124" s="7"/>
       <c r="K124" s="7"/>
       <c r="L124" s="7"/>
+      <c r="M124" s="7"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="4" t="n">
@@ -4159,6 +4356,7 @@
       <c r="J125" s="7"/>
       <c r="K125" s="7"/>
       <c r="L125" s="7"/>
+      <c r="M125" s="7"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="4" t="n">
@@ -4175,6 +4373,7 @@
       <c r="J126" s="7"/>
       <c r="K126" s="7"/>
       <c r="L126" s="7"/>
+      <c r="M126" s="7"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="4" t="n">
@@ -4191,6 +4390,7 @@
       <c r="J127" s="7"/>
       <c r="K127" s="7"/>
       <c r="L127" s="7"/>
+      <c r="M127" s="7"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="4" t="n">
@@ -4207,6 +4407,7 @@
       <c r="J128" s="7"/>
       <c r="K128" s="7"/>
       <c r="L128" s="7"/>
+      <c r="M128" s="7"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="4" t="n">
@@ -4223,6 +4424,7 @@
       <c r="J129" s="7"/>
       <c r="K129" s="7"/>
       <c r="L129" s="7"/>
+      <c r="M129" s="7"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="4" t="n">
@@ -4239,6 +4441,7 @@
       <c r="J130" s="7"/>
       <c r="K130" s="7"/>
       <c r="L130" s="7"/>
+      <c r="M130" s="7"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="4" t="n">
@@ -4255,6 +4458,7 @@
       <c r="J131" s="7"/>
       <c r="K131" s="7"/>
       <c r="L131" s="7"/>
+      <c r="M131" s="7"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="4" t="n">
@@ -4271,6 +4475,7 @@
       <c r="J132" s="7"/>
       <c r="K132" s="7"/>
       <c r="L132" s="7"/>
+      <c r="M132" s="7"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="4" t="n">
@@ -4287,6 +4492,7 @@
       <c r="J133" s="7"/>
       <c r="K133" s="7"/>
       <c r="L133" s="7"/>
+      <c r="M133" s="7"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="4" t="n">
@@ -4303,6 +4509,7 @@
       <c r="J134" s="7"/>
       <c r="K134" s="7"/>
       <c r="L134" s="7"/>
+      <c r="M134" s="7"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="4" t="n">
@@ -4319,6 +4526,7 @@
       <c r="J135" s="7"/>
       <c r="K135" s="7"/>
       <c r="L135" s="7"/>
+      <c r="M135" s="7"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="4" t="n">
@@ -4335,6 +4543,7 @@
       <c r="J136" s="7"/>
       <c r="K136" s="7"/>
       <c r="L136" s="7"/>
+      <c r="M136" s="7"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="4" t="n">
@@ -4351,6 +4560,7 @@
       <c r="J137" s="7"/>
       <c r="K137" s="7"/>
       <c r="L137" s="7"/>
+      <c r="M137" s="7"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="4" t="n">
@@ -4367,6 +4577,7 @@
       <c r="J138" s="7"/>
       <c r="K138" s="7"/>
       <c r="L138" s="7"/>
+      <c r="M138" s="7"/>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="4" t="n">
@@ -4383,6 +4594,7 @@
       <c r="J139" s="7"/>
       <c r="K139" s="7"/>
       <c r="L139" s="7"/>
+      <c r="M139" s="7"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="4" t="n">
@@ -4399,6 +4611,7 @@
       <c r="J140" s="7"/>
       <c r="K140" s="7"/>
       <c r="L140" s="7"/>
+      <c r="M140" s="7"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="4" t="n">
@@ -4415,6 +4628,7 @@
       <c r="J141" s="7"/>
       <c r="K141" s="7"/>
       <c r="L141" s="7"/>
+      <c r="M141" s="7"/>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="4" t="n">
@@ -4431,6 +4645,7 @@
       <c r="J142" s="7"/>
       <c r="K142" s="7"/>
       <c r="L142" s="7"/>
+      <c r="M142" s="7"/>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="4" t="n">
@@ -4447,6 +4662,7 @@
       <c r="J143" s="7"/>
       <c r="K143" s="7"/>
       <c r="L143" s="7"/>
+      <c r="M143" s="7"/>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="4" t="n">
@@ -4463,6 +4679,7 @@
       <c r="J144" s="7"/>
       <c r="K144" s="7"/>
       <c r="L144" s="7"/>
+      <c r="M144" s="7"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="4" t="n">
@@ -4479,6 +4696,7 @@
       <c r="J145" s="7"/>
       <c r="K145" s="7"/>
       <c r="L145" s="7"/>
+      <c r="M145" s="7"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="4" t="n">
@@ -4495,6 +4713,7 @@
       <c r="J146" s="7"/>
       <c r="K146" s="7"/>
       <c r="L146" s="7"/>
+      <c r="M146" s="7"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="4" t="n">
@@ -4511,6 +4730,7 @@
       <c r="J147" s="7"/>
       <c r="K147" s="7"/>
       <c r="L147" s="7"/>
+      <c r="M147" s="7"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="4" t="n">
@@ -4527,6 +4747,7 @@
       <c r="J148" s="7"/>
       <c r="K148" s="7"/>
       <c r="L148" s="7"/>
+      <c r="M148" s="7"/>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="4" t="n">
@@ -4543,6 +4764,7 @@
       <c r="J149" s="7"/>
       <c r="K149" s="7"/>
       <c r="L149" s="7"/>
+      <c r="M149" s="7"/>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="4" t="n">
@@ -4559,6 +4781,7 @@
       <c r="J150" s="7"/>
       <c r="K150" s="7"/>
       <c r="L150" s="7"/>
+      <c r="M150" s="7"/>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="4" t="n">
@@ -4575,6 +4798,7 @@
       <c r="J151" s="7"/>
       <c r="K151" s="7"/>
       <c r="L151" s="7"/>
+      <c r="M151" s="7"/>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="4" t="n">
@@ -4591,6 +4815,7 @@
       <c r="J152" s="7"/>
       <c r="K152" s="7"/>
       <c r="L152" s="7"/>
+      <c r="M152" s="7"/>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="4" t="n">
@@ -4607,6 +4832,7 @@
       <c r="J153" s="7"/>
       <c r="K153" s="7"/>
       <c r="L153" s="7"/>
+      <c r="M153" s="7"/>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="4" t="n">
@@ -4623,6 +4849,7 @@
       <c r="J154" s="7"/>
       <c r="K154" s="7"/>
       <c r="L154" s="7"/>
+      <c r="M154" s="7"/>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="4" t="n">
@@ -4639,6 +4866,7 @@
       <c r="J155" s="7"/>
       <c r="K155" s="7"/>
       <c r="L155" s="7"/>
+      <c r="M155" s="7"/>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="4" t="n">
@@ -4655,6 +4883,7 @@
       <c r="J156" s="7"/>
       <c r="K156" s="7"/>
       <c r="L156" s="7"/>
+      <c r="M156" s="7"/>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="4" t="n">
@@ -4671,6 +4900,7 @@
       <c r="J157" s="7"/>
       <c r="K157" s="7"/>
       <c r="L157" s="7"/>
+      <c r="M157" s="7"/>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="4" t="n">
@@ -4687,6 +4917,7 @@
       <c r="J158" s="7"/>
       <c r="K158" s="7"/>
       <c r="L158" s="7"/>
+      <c r="M158" s="7"/>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="4" t="n">
@@ -4703,6 +4934,7 @@
       <c r="J159" s="7"/>
       <c r="K159" s="7"/>
       <c r="L159" s="7"/>
+      <c r="M159" s="7"/>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="4" t="n">
@@ -4719,6 +4951,7 @@
       <c r="J160" s="7"/>
       <c r="K160" s="7"/>
       <c r="L160" s="7"/>
+      <c r="M160" s="7"/>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="4" t="n">
@@ -4735,6 +4968,7 @@
       <c r="J161" s="7"/>
       <c r="K161" s="7"/>
       <c r="L161" s="7"/>
+      <c r="M161" s="7"/>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="4" t="n">
@@ -4751,6 +4985,7 @@
       <c r="J162" s="7"/>
       <c r="K162" s="7"/>
       <c r="L162" s="7"/>
+      <c r="M162" s="7"/>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="4" t="n">
@@ -4767,6 +5002,7 @@
       <c r="J163" s="7"/>
       <c r="K163" s="7"/>
       <c r="L163" s="7"/>
+      <c r="M163" s="7"/>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="4" t="n">
@@ -4783,6 +5019,7 @@
       <c r="J164" s="7"/>
       <c r="K164" s="7"/>
       <c r="L164" s="7"/>
+      <c r="M164" s="7"/>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="4" t="n">
@@ -4799,6 +5036,7 @@
       <c r="J165" s="7"/>
       <c r="K165" s="7"/>
       <c r="L165" s="7"/>
+      <c r="M165" s="7"/>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="4" t="n">
@@ -4815,6 +5053,7 @@
       <c r="J166" s="7"/>
       <c r="K166" s="7"/>
       <c r="L166" s="7"/>
+      <c r="M166" s="7"/>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="4" t="n">
@@ -4831,6 +5070,7 @@
       <c r="J167" s="7"/>
       <c r="K167" s="7"/>
       <c r="L167" s="7"/>
+      <c r="M167" s="7"/>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="4" t="n">
@@ -4847,6 +5087,7 @@
       <c r="J168" s="7"/>
       <c r="K168" s="7"/>
       <c r="L168" s="7"/>
+      <c r="M168" s="7"/>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="4" t="n">
@@ -4863,6 +5104,7 @@
       <c r="J169" s="7"/>
       <c r="K169" s="7"/>
       <c r="L169" s="7"/>
+      <c r="M169" s="7"/>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="4" t="n">
@@ -4879,6 +5121,7 @@
       <c r="J170" s="7"/>
       <c r="K170" s="7"/>
       <c r="L170" s="7"/>
+      <c r="M170" s="7"/>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="4" t="n">
@@ -4895,6 +5138,7 @@
       <c r="J171" s="7"/>
       <c r="K171" s="7"/>
       <c r="L171" s="7"/>
+      <c r="M171" s="7"/>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="4" t="n">
@@ -4911,6 +5155,7 @@
       <c r="J172" s="7"/>
       <c r="K172" s="7"/>
       <c r="L172" s="7"/>
+      <c r="M172" s="7"/>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="4" t="n">
@@ -4927,6 +5172,7 @@
       <c r="J173" s="7"/>
       <c r="K173" s="7"/>
       <c r="L173" s="7"/>
+      <c r="M173" s="7"/>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="4" t="n">
@@ -4943,6 +5189,7 @@
       <c r="J174" s="7"/>
       <c r="K174" s="7"/>
       <c r="L174" s="7"/>
+      <c r="M174" s="7"/>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="4" t="n">
@@ -4959,6 +5206,7 @@
       <c r="J175" s="7"/>
       <c r="K175" s="7"/>
       <c r="L175" s="7"/>
+      <c r="M175" s="7"/>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="4" t="n">
@@ -4975,6 +5223,7 @@
       <c r="J176" s="7"/>
       <c r="K176" s="7"/>
       <c r="L176" s="7"/>
+      <c r="M176" s="7"/>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="4" t="n">
@@ -4991,6 +5240,7 @@
       <c r="J177" s="7"/>
       <c r="K177" s="7"/>
       <c r="L177" s="7"/>
+      <c r="M177" s="7"/>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="4" t="n">
@@ -5007,6 +5257,7 @@
       <c r="J178" s="7"/>
       <c r="K178" s="7"/>
       <c r="L178" s="7"/>
+      <c r="M178" s="7"/>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="4" t="n">
@@ -5023,6 +5274,7 @@
       <c r="J179" s="7"/>
       <c r="K179" s="7"/>
       <c r="L179" s="7"/>
+      <c r="M179" s="7"/>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="4" t="n">
@@ -5039,6 +5291,7 @@
       <c r="J180" s="7"/>
       <c r="K180" s="7"/>
       <c r="L180" s="7"/>
+      <c r="M180" s="7"/>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="4" t="n">
@@ -5055,6 +5308,7 @@
       <c r="J181" s="7"/>
       <c r="K181" s="7"/>
       <c r="L181" s="7"/>
+      <c r="M181" s="7"/>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="4" t="n">
@@ -5071,6 +5325,7 @@
       <c r="J182" s="7"/>
       <c r="K182" s="7"/>
       <c r="L182" s="7"/>
+      <c r="M182" s="7"/>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="4" t="n">
@@ -5087,6 +5342,7 @@
       <c r="J183" s="7"/>
       <c r="K183" s="7"/>
       <c r="L183" s="7"/>
+      <c r="M183" s="7"/>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="4" t="n">
@@ -5103,6 +5359,7 @@
       <c r="J184" s="7"/>
       <c r="K184" s="7"/>
       <c r="L184" s="7"/>
+      <c r="M184" s="7"/>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="4" t="n">
@@ -5119,6 +5376,7 @@
       <c r="J185" s="7"/>
       <c r="K185" s="7"/>
       <c r="L185" s="7"/>
+      <c r="M185" s="7"/>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="4" t="n">
@@ -5135,6 +5393,7 @@
       <c r="J186" s="7"/>
       <c r="K186" s="7"/>
       <c r="L186" s="7"/>
+      <c r="M186" s="7"/>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="4" t="n">
@@ -5151,6 +5410,7 @@
       <c r="J187" s="7"/>
       <c r="K187" s="7"/>
       <c r="L187" s="7"/>
+      <c r="M187" s="7"/>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="4" t="n">
@@ -5167,6 +5427,7 @@
       <c r="J188" s="7"/>
       <c r="K188" s="7"/>
       <c r="L188" s="7"/>
+      <c r="M188" s="7"/>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="4" t="n">
@@ -5183,6 +5444,7 @@
       <c r="J189" s="7"/>
       <c r="K189" s="7"/>
       <c r="L189" s="7"/>
+      <c r="M189" s="7"/>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="4" t="n">
@@ -5199,6 +5461,7 @@
       <c r="J190" s="7"/>
       <c r="K190" s="7"/>
       <c r="L190" s="7"/>
+      <c r="M190" s="7"/>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="4" t="n">
@@ -5215,6 +5478,7 @@
       <c r="J191" s="7"/>
       <c r="K191" s="7"/>
       <c r="L191" s="7"/>
+      <c r="M191" s="7"/>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="4" t="n">
@@ -5231,6 +5495,7 @@
       <c r="J192" s="7"/>
       <c r="K192" s="7"/>
       <c r="L192" s="7"/>
+      <c r="M192" s="7"/>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="4" t="n">
@@ -5247,6 +5512,7 @@
       <c r="J193" s="7"/>
       <c r="K193" s="7"/>
       <c r="L193" s="7"/>
+      <c r="M193" s="7"/>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="4" t="n">
@@ -5263,6 +5529,7 @@
       <c r="J194" s="7"/>
       <c r="K194" s="7"/>
       <c r="L194" s="7"/>
+      <c r="M194" s="7"/>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="4" t="n">
@@ -5279,6 +5546,7 @@
       <c r="J195" s="7"/>
       <c r="K195" s="7"/>
       <c r="L195" s="7"/>
+      <c r="M195" s="7"/>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="4" t="n">
@@ -5295,6 +5563,7 @@
       <c r="J196" s="7"/>
       <c r="K196" s="7"/>
       <c r="L196" s="7"/>
+      <c r="M196" s="7"/>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="4" t="n">
@@ -5311,6 +5580,7 @@
       <c r="J197" s="7"/>
       <c r="K197" s="7"/>
       <c r="L197" s="7"/>
+      <c r="M197" s="7"/>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="4" t="n">
@@ -5327,6 +5597,7 @@
       <c r="J198" s="7"/>
       <c r="K198" s="7"/>
       <c r="L198" s="7"/>
+      <c r="M198" s="7"/>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="4" t="n">
@@ -5343,6 +5614,7 @@
       <c r="J199" s="7"/>
       <c r="K199" s="7"/>
       <c r="L199" s="7"/>
+      <c r="M199" s="7"/>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="4" t="n">
@@ -5359,6 +5631,7 @@
       <c r="J200" s="7"/>
       <c r="K200" s="7"/>
       <c r="L200" s="7"/>
+      <c r="M200" s="7"/>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="4" t="n">
@@ -5375,6 +5648,7 @@
       <c r="J201" s="7"/>
       <c r="K201" s="7"/>
       <c r="L201" s="7"/>
+      <c r="M201" s="7"/>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="4" t="n">
@@ -5391,6 +5665,7 @@
       <c r="J202" s="7"/>
       <c r="K202" s="7"/>
       <c r="L202" s="7"/>
+      <c r="M202" s="7"/>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="4" t="n">
@@ -5407,6 +5682,7 @@
       <c r="J203" s="7"/>
       <c r="K203" s="7"/>
       <c r="L203" s="7"/>
+      <c r="M203" s="7"/>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="4" t="n">
@@ -5423,6 +5699,7 @@
       <c r="J204" s="7"/>
       <c r="K204" s="7"/>
       <c r="L204" s="7"/>
+      <c r="M204" s="7"/>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="4" t="n">
@@ -5439,9 +5716,10 @@
       <c r="J205" s="7"/>
       <c r="K205" s="7"/>
       <c r="L205" s="7"/>
+      <c r="M205" s="7"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="7">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D205" type="list">
       <formula1>Components!$A$5:$A$20</formula1>
       <formula2>0</formula2>
@@ -5458,11 +5736,15 @@
       <formula1>"A step of the argument collapses,A claim must be weakened,One footnote dies,No effect on the argument"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L5:L205" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K205" type="list">
+      <formula1>"author,author chose from assistant's options,assistant,not yet decided"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M5:M205" type="list">
       <formula1>"Pre-release,Post-release"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K205" type="whole">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L5:L205" type="whole">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5495,233 +5777,233 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B16" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E16" s="6" t="s">
         <v>97</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5754,7 +6036,7 @@
     </row>
     <row r="22" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B22" s="11"/>
       <c r="C22" s="11"/>
@@ -5790,158 +6072,158 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C16" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C19" s="4"/>
     </row>
@@ -5983,37 +6265,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -6024,10 +6306,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -6038,10 +6320,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -6052,10 +6334,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="12"/>
@@ -6066,10 +6348,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
@@ -6080,10 +6362,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -6094,10 +6376,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -6108,10 +6390,10 @@
     </row>
     <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
@@ -6122,10 +6404,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C13" s="3" t="n">
         <f aca="false">SUM(C5:C12)</f>
@@ -6138,7 +6420,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E14" s="16" t="str">
         <f aca="false">IF(E13=0,"",IF(E12="",0,E12/E13))</f>
@@ -6147,7 +6429,7 @@
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B16" s="11"/>
       <c r="C16" s="11"/>
@@ -6156,7 +6438,7 @@
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -6165,7 +6447,7 @@
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
@@ -6206,12 +6488,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6219,19 +6501,19 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6239,16 +6521,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F5" s="4"/>
     </row>
@@ -6257,16 +6539,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F6" s="4"/>
     </row>
@@ -6275,16 +6557,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F7" s="4"/>
     </row>
@@ -6293,16 +6575,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>179</v>
-      </c>
       <c r="D8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F8" s="4"/>
     </row>
@@ -6311,16 +6593,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F9" s="4"/>
     </row>
@@ -6329,16 +6611,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F10" s="4"/>
     </row>
@@ -6347,19 +6629,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>186</v>
-      </c>
       <c r="D11" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6367,16 +6649,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F12" s="4"/>
     </row>
@@ -6385,16 +6667,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F13" s="4"/>
     </row>
@@ -6403,16 +6685,16 @@
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F14" s="4"/>
     </row>
@@ -6421,16 +6703,16 @@
         <v>11</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F15" s="4"/>
     </row>
@@ -6439,16 +6721,16 @@
         <v>12</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F16" s="4"/>
     </row>
@@ -6457,16 +6739,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F17" s="4"/>
     </row>
@@ -6475,16 +6757,16 @@
         <v>14</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F18" s="4"/>
     </row>
@@ -6493,16 +6775,16 @@
         <v>15</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F19" s="4"/>
     </row>
@@ -6511,19 +6793,19 @@
         <v>16</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6531,19 +6813,19 @@
         <v>17</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6551,16 +6833,16 @@
         <v>18</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F22" s="4"/>
     </row>
@@ -6569,16 +6851,16 @@
         <v>19</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F23" s="4"/>
     </row>
@@ -6587,19 +6869,19 @@
         <v>20</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6607,16 +6889,16 @@
         <v>21</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F25" s="4"/>
     </row>
@@ -6625,16 +6907,16 @@
         <v>22</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F26" s="4"/>
     </row>
@@ -6643,19 +6925,19 @@
         <v>23</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6663,19 +6945,19 @@
         <v>24</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C28" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="F28" s="4" t="s">
         <v>234</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6683,22 +6965,22 @@
         <v>25</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F29" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="17" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B31" s="17"/>
       <c r="C31" s="17"/>
@@ -6708,7 +6990,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="17" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="17"/>
@@ -6752,181 +7034,181 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I9" s="6"/>
     </row>

</xml_diff>

<commit_message>
v1.8: act on the review of 9d4ab14/26a0b7b (undecided markers, unknown phase, headers, example phase notes, docs)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C2RNJLwLc4CBTFwfe5m9zY
</commit_message>
<xml_diff>
--- a/kit/citation-provenance-kit.xlsx
+++ b/kit/citation-provenance-kit.xlsx
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="280">
   <si>
     <t xml:space="preserve">Citation provenance kit — reproduction kit</t>
   </si>
@@ -154,7 +154,7 @@
     <t xml:space="preserve">Columns the original log lacked</t>
   </si>
   <si>
-    <t xml:space="preserve">The original log kept three things for each entry: what was wrong, what was right, and how it came to notice (Appendix A-0). Every other column here was added afterwards. The paper says the six fields of §7-1 were recorded for each correction (§7-1, §8-1); the published log (Appendix A-2, A-6) shows no 'what would have happened' column.
+    <t xml:space="preserve">Besides its numbering, the original log kept three things for each entry: what was wrong, what was right, and how it came to notice (Appendix A-0). The component and rule columns were added afterwards, at grade D. The paper says the six fields of §7-1 were recorded for each correction, and §8-1 that the corrections were logged with their component, rule and consequence; the published log (Appendix A-2, and A-6 in paper v1.2) shows no 'what would have happened' column.
 'Did an existing rule fire?': two rules failed to prevent their own failure from recurring, and the log could not show it (Appendix B, §9-1).
 'Duration': no effort was recorded and it cannot be reconstructed (§8-1).
 'Stakes': the distinction between a step of the argument collapsing and one footnote dying (§7-1), as a filterable field.
@@ -506,9 +506,6 @@
   </si>
   <si>
     <t xml:space="preserve">A step of the argument collapses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">author</t>
   </si>
   <si>
     <t xml:space="preserve">Pre-release</t>
@@ -2163,7 +2160,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="225" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
@@ -2310,12 +2307,10 @@
       <c r="J5" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="K5" s="6" t="s">
-        <v>43</v>
-      </c>
+      <c r="K5" s="6"/>
       <c r="L5" s="6"/>
       <c r="M5" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5777,29 +5772,29 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="C4" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5807,203 +5802,203 @@
         <v>36</v>
       </c>
       <c r="B5" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="C6" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>59</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="C7" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>63</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="C8" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>67</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="C9" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>72</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="C10" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>76</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="C11" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>80</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="C12" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="C13" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="4" t="s">
         <v>88</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B14" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="C14" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>92</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="C15" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="D15" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E15" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="C16" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="C16" s="6" t="s">
-        <v>100</v>
-      </c>
       <c r="D16" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6036,7 +6031,7 @@
     </row>
     <row r="22" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B22" s="11"/>
       <c r="C22" s="11"/>
@@ -6072,158 +6067,158 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="8" t="s">
         <v>105</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="9" t="s">
         <v>108</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="9" t="s">
         <v>111</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="9" t="s">
         <v>114</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="9" t="s">
         <v>117</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>119</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>121</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>122</v>
       </c>
       <c r="C11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>123</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>124</v>
       </c>
       <c r="C12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>125</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>126</v>
       </c>
       <c r="C13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>127</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>128</v>
       </c>
       <c r="C14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>129</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>130</v>
       </c>
       <c r="C15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>131</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>132</v>
       </c>
       <c r="C16" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>133</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>134</v>
       </c>
       <c r="C17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>135</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>136</v>
       </c>
       <c r="C18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>137</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>138</v>
       </c>
       <c r="C19" s="4"/>
     </row>
@@ -6265,37 +6260,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="C4" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>144</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>146</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>147</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
@@ -6306,10 +6301,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>148</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>149</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
@@ -6320,10 +6315,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>150</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>151</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
@@ -6334,10 +6329,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>152</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>153</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="12"/>
@@ -6348,10 +6343,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>154</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>155</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
@@ -6362,10 +6357,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>156</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>157</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -6376,10 +6371,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>158</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>159</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -6390,10 +6385,10 @@
     </row>
     <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>160</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>161</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
@@ -6404,10 +6399,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B13" s="14" t="s">
         <v>162</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>163</v>
       </c>
       <c r="C13" s="3" t="n">
         <f aca="false">SUM(C5:C12)</f>
@@ -6420,7 +6415,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E14" s="16" t="str">
         <f aca="false">IF(E13=0,"",IF(E12="",0,E12/E13))</f>
@@ -6429,7 +6424,7 @@
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B16" s="11"/>
       <c r="C16" s="11"/>
@@ -6438,7 +6433,7 @@
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -6447,7 +6442,7 @@
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
@@ -6488,12 +6483,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6501,19 +6496,19 @@
         <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>173</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6521,16 +6516,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>177</v>
-      </c>
       <c r="E5" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F5" s="4"/>
     </row>
@@ -6539,16 +6534,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>179</v>
-      </c>
       <c r="D6" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F6" s="4"/>
     </row>
@@ -6557,16 +6552,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>180</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>181</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>36</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F7" s="4"/>
     </row>
@@ -6575,16 +6570,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>36</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F8" s="4"/>
     </row>
@@ -6593,16 +6588,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>185</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>186</v>
       </c>
       <c r="F9" s="4"/>
     </row>
@@ -6611,16 +6606,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>188</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>189</v>
       </c>
       <c r="F10" s="4"/>
     </row>
@@ -6629,19 +6624,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>36</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6649,16 +6644,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>194</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>195</v>
       </c>
       <c r="F12" s="4"/>
     </row>
@@ -6667,16 +6662,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>198</v>
-      </c>
       <c r="E13" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F13" s="4"/>
     </row>
@@ -6685,16 +6680,16 @@
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>199</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>200</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>36</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F14" s="4"/>
     </row>
@@ -6703,16 +6698,16 @@
         <v>11</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="D15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>202</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>203</v>
       </c>
       <c r="F15" s="4"/>
     </row>
@@ -6721,16 +6716,16 @@
         <v>12</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>205</v>
-      </c>
       <c r="D16" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F16" s="4"/>
     </row>
@@ -6739,16 +6734,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F17" s="4"/>
     </row>
@@ -6757,16 +6752,16 @@
         <v>14</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>208</v>
-      </c>
       <c r="D18" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F18" s="4"/>
     </row>
@@ -6775,16 +6770,16 @@
         <v>15</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F19" s="4"/>
     </row>
@@ -6793,19 +6788,19 @@
         <v>16</v>
       </c>
       <c r="B20" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>210</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>211</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>36</v>
       </c>
       <c r="E20" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="F20" s="4" t="s">
         <v>212</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6813,19 +6808,19 @@
         <v>17</v>
       </c>
       <c r="B21" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="C21" s="4" t="s">
-        <v>215</v>
-      </c>
       <c r="D21" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6833,16 +6828,16 @@
         <v>18</v>
       </c>
       <c r="B22" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="D22" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E22" s="4" t="s">
         <v>217</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>218</v>
       </c>
       <c r="F22" s="4"/>
     </row>
@@ -6851,16 +6846,16 @@
         <v>19</v>
       </c>
       <c r="B23" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>219</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>220</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>36</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F23" s="4"/>
     </row>
@@ -6869,19 +6864,19 @@
         <v>20</v>
       </c>
       <c r="B24" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>222</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>223</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>36</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6889,16 +6884,16 @@
         <v>21</v>
       </c>
       <c r="B25" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="D25" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="D25" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="E25" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F25" s="4"/>
     </row>
@@ -6907,16 +6902,16 @@
         <v>22</v>
       </c>
       <c r="B26" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="D26" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="E26" s="4" t="s">
         <v>230</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>231</v>
       </c>
       <c r="F26" s="4"/>
     </row>
@@ -6925,19 +6920,19 @@
         <v>23</v>
       </c>
       <c r="B27" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="E27" s="4" t="s">
+      <c r="F27" s="4" t="s">
         <v>233</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6945,19 +6940,19 @@
         <v>24</v>
       </c>
       <c r="B28" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="C28" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="D28" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="D28" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>237</v>
-      </c>
       <c r="F28" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6965,22 +6960,22 @@
         <v>25</v>
       </c>
       <c r="B29" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>239</v>
-      </c>
       <c r="D29" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F29" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="17" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B31" s="17"/>
       <c r="C31" s="17"/>
@@ -6990,7 +6985,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="17" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="17"/>
@@ -7034,181 +7029,181 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="H4" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="I4" s="5" t="s">
         <v>250</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="I5" s="6" t="s">
         <v>258</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="G6" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>263</v>
-      </c>
       <c r="H6" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="G7" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="G7" s="6" t="s">
+      <c r="H7" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="I7" s="6" t="s">
         <v>268</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C8" s="6" t="s">
+      <c r="D8" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="G8" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="G8" s="6" t="s">
+      <c r="H8" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="C9" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="G9" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>280</v>
-      </c>
       <c r="H9" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I9" s="6"/>
     </row>

</xml_diff>

<commit_message>
Kit v1.10 (unreleased): derived documents and the editions they were made from
Add tools/derivedcheck.py, register/derived.jsonl, schema/derived.schema.json
and tests. Record the current editions of both papers in the status log.
Say that the kit was made for the paper's v1.1 and that files made from v1.2
name it; list tags with the date they were seen; bump the workbook's label,
which v1.9 left at 1.8.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Eoppy7WpRmSWDgHU6JWiT4
</commit_message>
<xml_diff>
--- a/kit/citation-provenance-kit.xlsx
+++ b/kit/citation-provenance-kit.xlsx
@@ -117,7 +117,7 @@
     <t xml:space="preserve">Citation provenance kit — reproduction kit</t>
   </si>
   <si>
-    <t xml:space="preserve">Kit v1.8 · accompanies What Breaks in a Citation, v1.1 (26 July 2026) · CC0 1.0 (no rights reserved)</t>
+    <t xml:space="preserve">Kit v1.10 · accompanies What Breaks in a Citation, v1.1 (26 July 2026); files made from v1.2 (12 October 2026) name it · CC0 1.0 (no rights reserved)</t>
   </si>
   <si>
     <t xml:space="preserve">What this is</t>
@@ -177,7 +177,7 @@
     <t xml:space="preserve">Source papers</t>
   </si>
   <si>
-    <t xml:space="preserve">What Breaks in a Citation (EN) https://lnkd.in/p/giTfeMUh · (JA) https://lnkd.in/p/gFUXFv2w
+    <t xml:space="preserve">What Breaks in a Citation — links listed since kit v1.0: (EN) https://lnkd.in/p/giTfeMUh · (JA) https://lnkd.in/p/gFUXFv2w; v1.2, as cited in Hypothetical Technical Blog #28: (EN) https://lnkd.in/p/gjQ2RAPW · (JA) https://lnkd.in/p/gW5xwpFK
 What Your Buyer Is Defending Against (EN) https://lnkd.in/p/gHNjBuCd · (JA) https://lnkd.in/p/gF-kd9DF</t>
   </si>
   <si>
@@ -2184,7 +2184,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
         <v>16</v>
       </c>

</xml_diff>

<commit_message>
Kit v1.11 (draft): the 1.6% ratio is the judgment's (#76); workbook row on the marker (#77); READMEs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017nRQoJfYS1HKcabqfT7Nan
</commit_message>
<xml_diff>
--- a/kit/citation-provenance-kit.xlsx
+++ b/kit/citation-provenance-kit.xlsx
@@ -117,7 +117,7 @@
     <t xml:space="preserve">Citation provenance kit — reproduction kit</t>
   </si>
   <si>
-    <t xml:space="preserve">Kit v1.10 · accompanies What Breaks in a Citation, v1.1 (26 July 2026); files made from v1.2 (12 October 2026) name it · CC0 1.0 (no rights reserved)</t>
+    <t xml:space="preserve">Kit v1.11 · accompanies What Breaks in a Citation, v1.1 (26 July 2026); files made from v1.2 (12 October 2026) name it · CC0 1.0 (no rights reserved)</t>
   </si>
   <si>
     <t xml:space="preserve">What this is</t>
@@ -874,10 +874,10 @@
     <t xml:space="preserve">Declare every component and grade token in the document that uses it. An undefined token reached publication in the source project (§7-4).</t>
   </si>
   <si>
-    <t xml:space="preserve">Derived values (provisional, untested)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A value computed from cited primaries is neither A nor D. The paper proposes a marker but has not tested one (§4-6, §9-3). Suggested interim: grade the operands, and state the arithmetic beside it, labelled as the author's.</t>
+    <t xml:space="preserve">Derived values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A value computed from cited primaries is neither A nor D (§4-6, §9-3). §4-6 says the paper proposes a provisional marker; none appears in it (entry #77 of the author's log after v1.2). Grade the operands and state who did the arithmetic: [operands: A | arithmetic: author]. Record the value, its inputs and the operation in register/computed.jsonl and check it with tools/calccheck.py (kit v1.11). Check first whether the source states the value itself: the paper's own example, about 1.6%, is stated in the judgment (#76).</t>
   </si>
   <si>
     <t xml:space="preserve">Cost calculator — a method, not a number</t>

</xml_diff>

<commit_message>
Kit v1.11 (draft): review fixes to calccheck, register and READMEs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017nRQoJfYS1HKcabqfT7Nan
</commit_message>
<xml_diff>
--- a/kit/citation-provenance-kit.xlsx
+++ b/kit/citation-provenance-kit.xlsx
@@ -577,7 +577,7 @@
     <t xml:space="preserve">No (derived values: see Grades sheet)</t>
   </si>
   <si>
-    <t xml:space="preserve">A 1.6% ratio derived from two cited primary values; never examined in v1.1.</t>
+    <t xml:space="preserve">'May 2027', the author's arithmetic on a period (#35). The 1.6% ratio, once listed here as derived from two cited primary values, is stated in the judgment (#76).</t>
   </si>
   <si>
     <t xml:space="preserve">page</t>
@@ -877,7 +877,7 @@
     <t xml:space="preserve">Derived values</t>
   </si>
   <si>
-    <t xml:space="preserve">A value computed from cited primaries is neither A nor D (§4-6, §9-3). §4-6 says the paper proposes a provisional marker; none appears in it (entry #77 of the author's log after v1.2). Grade the operands and state who did the arithmetic: [operands: A | arithmetic: author]. Record the value, its inputs and the operation in register/computed.jsonl and check it with tools/calccheck.py (kit v1.11). Check first whether the source states the value itself: the paper's own example, about 1.6%, is stated in the judgment (#76).</t>
+    <t xml:space="preserve">A value computed from cited primaries is neither A nor D (§4-6, §9-3). §4-6 says the paper proposes a provisional marker; none appears in it (entry #77 of the author's log after v1.2). Grade the operands and say whose the arithmetic is, within the closed vocabulary: [figure: A | attribution: D]. Record the value, its inputs and the operation in register/computed.jsonl and check it with tools/calccheck.py (kit v1.11). Check first whether the source states the value itself: the paper's own example, about 1.6%, is stated in the judgment (#76).</t>
   </si>
   <si>
     <t xml:space="preserve">Cost calculator — a method, not a number</t>
@@ -5814,7 +5814,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>55</v>
       </c>

</xml_diff>

<commit_message>
Kit v1.12 (in preparation): identifiers, namespaces and idcheck
Adds tools/idcheck.py, register/namespaces.json, register/identifiers.jsonl,
two schemas, tests and evidence. Both READMEs now name the namespace of
every number they write (Blog #N, log #N / ログ#N); components.csv and the
workbook say log #22. Not released.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012GHKTPrv7gqJNPJ7Qn8DDG
</commit_message>
<xml_diff>
--- a/kit/citation-provenance-kit.xlsx
+++ b/kit/citation-provenance-kit.xlsx
@@ -117,7 +117,7 @@
     <t xml:space="preserve">Citation provenance kit — reproduction kit</t>
   </si>
   <si>
-    <t xml:space="preserve">Kit v1.11 · accompanies What Breaks in a Citation, v1.1 (26 July 2026); files made from v1.2 (12 October 2026) name it · CC0 1.0 (no rights reserved)</t>
+    <t xml:space="preserve">Kit v1.12 · accompanies What Breaks in a Citation, v1.1 (26 July 2026); files made from v1.2 (12 October 2026) name it · CC0 1.0 (no rights reserved)</t>
   </si>
   <si>
     <t xml:space="preserve">What this is</t>
@@ -628,7 +628,7 @@
     <t xml:space="preserve">The identifier resolves to the one instrument intended, not a namesake.</t>
   </si>
   <si>
-    <t xml:space="preserve">G.S.R. 206(E) of 2015 and of 2021 (#22).</t>
+    <t xml:space="preserve">G.S.R. 206(E) of 2015 and of 2021 (log #22). Write the namespace with the number: Blog #22 is a post. Check with tools/idcheck.py (kit v1.12).</t>
   </si>
   <si>
     <t xml:space="preserve">existence</t>

</xml_diff>

<commit_message>
Kit v1.12: fixes from the review of 233e072
Full-width digits, Japanese name boundaries, supersedes chains, deep
nesting, huge ranges, absent named numbers, URL fragments, dash key
values; register text names its numbers (three records superseded);
the Components column names the log throughout.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012GHKTPrv7gqJNPJ7Qn8DDG
</commit_message>
<xml_diff>
--- a/kit/citation-provenance-kit.xlsx
+++ b/kit/citation-provenance-kit.xlsx
@@ -562,7 +562,7 @@
     <t xml:space="preserve">No</t>
   </si>
   <si>
-    <t xml:space="preserve">A rule cited as listing 'life cycle cost' among its criteria; the phrase was not in it (#8).</t>
+    <t xml:space="preserve">A rule cited as listing 'life cycle cost' among its criteria; the phrase was not in it (log #8).</t>
   </si>
   <si>
     <t xml:space="preserve">figure</t>
@@ -577,7 +577,7 @@
     <t xml:space="preserve">No (derived values: see Grades sheet)</t>
   </si>
   <si>
-    <t xml:space="preserve">'May 2027', the author's arithmetic on a period (#35). The 1.6% ratio, once listed here as derived from two cited primary values, is stated in the judgment (#76).</t>
+    <t xml:space="preserve">'May 2027', the author's arithmetic on a period (log #35). The 1.6% ratio, once listed here as derived from two cited primary values, is stated in the judgment (log #76).</t>
   </si>
   <si>
     <t xml:space="preserve">page</t>
@@ -601,7 +601,7 @@
     <t xml:space="preserve">A date attributed to the source or computed from it is correct.</t>
   </si>
   <si>
-    <t xml:space="preserve">'Eighteen months from publication' rendered as a specific day (#11).</t>
+    <t xml:space="preserve">'Eighteen months from publication' rendered as a specific day (log #11).</t>
   </si>
   <si>
     <t xml:space="preserve">edition</t>
@@ -616,7 +616,7 @@
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
-    <t xml:space="preserve">Two vintages of an official translation in circulation (#5); the change-marked edition cited as authoritative (#23).</t>
+    <t xml:space="preserve">Two vintages of an official translation in circulation (log #5); the change-marked edition cited as authoritative (log #23).</t>
   </si>
   <si>
     <t xml:space="preserve">identifier</t>
@@ -640,7 +640,7 @@
     <t xml:space="preserve">The cited provision or document exists in the version relied on.</t>
   </si>
   <si>
-    <t xml:space="preserve">A supplementary principle deleted in a code revision (#14); a memorandum absent from the consolidated rules (#9).</t>
+    <t xml:space="preserve">A supplementary principle deleted in a code revision (log #14); a memorandum absent from the consolidated rules (log #9).</t>
   </si>
   <si>
     <t xml:space="preserve">commencement</t>
@@ -652,7 +652,7 @@
     <t xml:space="preserve">The provision is in force on the date the text speaks from.</t>
   </si>
   <si>
-    <t xml:space="preserve">An obligation described in the present tense, eighteen months before commencement (#18, recurred #24).</t>
+    <t xml:space="preserve">An obligation described in the present tense, eighteen months before commencement (log #18; recurred as log #24).</t>
   </si>
   <si>
     <t xml:space="preserve">attribution</t>
@@ -664,7 +664,7 @@
     <t xml:space="preserve">The statement is attributed to the body that actually made it.</t>
   </si>
   <si>
-    <t xml:space="preserve">Guidance from a professional institute treated as if it settled a statutory question (#17).</t>
+    <t xml:space="preserve">Guidance from a professional institute treated as if it settled a statutory question (log #17).</t>
   </si>
   <si>
     <t xml:space="preserve">dependency</t>

</xml_diff>